<commit_message>
feat: round 11 — BMR/TDEE + coaching dashboard + DD-MM-YYYY dates
Profile ENERGY card (BMR/TDEE via Katch-McArdle/Mifflin) + Bio popup,
coach dashboard (adherence, body/energy, strength) reading athlete
bio/1RM via new program_state columns + RLS, DD-MM-YYYY date format,
and Excel program_type (general/powerlifting).

Fixes found during e2e:
- Save bio popup covered by bottom nav: .screen-enter kept a lingering
  transform (animation fill `both`), making .atlas-screen the containing
  block so the sheet backdrop no longer covered the full app. Switched
  fill-mode to `backwards` + capped sheet height.
- Setup Program required 1RM even for general programs (no weight calc):
  gate 1RM inputs/validation on programType, general needs only a date.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/atlaslog-program-template.xlsx
+++ b/apps/web/public/atlaslog-program-template.xlsx
@@ -903,7 +903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -929,9 +929,17 @@
         <v>Squat · Bench · Deadlift</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>program_type</v>
+      </c>
+      <c r="B4" t="str">
+        <v>powerlifting</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>